<commit_message>
change on the logic and the structure of the excel
</commit_message>
<xml_diff>
--- a/data/raw/gastos.xlsx
+++ b/data/raw/gastos.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="29">
   <si>
     <t xml:space="preserve">tipo</t>
   </si>
@@ -64,13 +64,13 @@
     <t xml:space="preserve">hbo</t>
   </si>
   <si>
-    <t xml:space="preserve">credito</t>
-  </si>
-  <si>
     <t xml:space="preserve">steam</t>
   </si>
   <si>
-    <t xml:space="preserve">prestamo nu</t>
+    <t xml:space="preserve">credito nu </t>
+  </si>
+  <si>
+    <t xml:space="preserve">regalo</t>
   </si>
   <si>
     <t xml:space="preserve">pantalla</t>
@@ -98,6 +98,15 @@
   </si>
   <si>
     <t xml:space="preserve">ahorro y fondo de emergencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">desarrollo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gimnasio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mensualidad de gimnasio</t>
   </si>
 </sst>
 </file>
@@ -181,7 +190,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -316,11 +325,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.93"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="25.51"/>
   </cols>
   <sheetData>
@@ -412,16 +421,16 @@
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>26300</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>11</v>
@@ -432,7 +441,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>17</v>
@@ -441,69 +450,89 @@
         <v>30700</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="1" t="n">
         <v>12000</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="G7" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D8" s="1" t="n">
         <v>11000</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G8" s="0" t="s">
+      <c r="G8" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="1" t="n">
         <v>200000</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mejoras en absolutizacion de rutas, logica de analisis
</commit_message>
<xml_diff>
--- a/data/raw/gastos.xlsx
+++ b/data/raw/gastos.xlsx
@@ -5,10 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Gastos_fijos" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Movimientos" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,101 +21,120 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="35">
+  <si>
+    <t xml:space="preserve">categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nombre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">descripcion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fecha_inicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fecha_fin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">frecuencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">entretenimiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spotify</t>
+  </si>
+  <si>
+    <t xml:space="preserve">suscripcion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mensual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">salida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hbo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">steam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">credito nu </t>
+  </si>
+  <si>
+    <t xml:space="preserve">18/03/2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valorant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25/09/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">regalo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pantalla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21/07/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18/12/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuentas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuota de manejo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuenta nu </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuenta bancolombia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mensual </t>
+  </si>
+  <si>
+    <t xml:space="preserve">finanzas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ahorro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ahorro y fondo de emergencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">desarrollo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gimnasio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mensualidad de gimnasio</t>
+  </si>
   <si>
     <t xml:space="preserve">tipo</t>
   </si>
   <si>
-    <t xml:space="preserve">categoria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nombre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">valor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">descripcion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fecha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">frecuencia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fijo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">entretenimiento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spotify</t>
-  </si>
-  <si>
-    <t xml:space="preserve">suscripcion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mensual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">salida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hbo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">steam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">credito nu </t>
-  </si>
-  <si>
-    <t xml:space="preserve">regalo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pantalla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuentas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuota de manejo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuenta nu </t>
-  </si>
-  <si>
-    <t xml:space="preserve">cuenta bancolombia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mensual </t>
-  </si>
-  <si>
-    <t xml:space="preserve">finanzas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ahorro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ahorro y fondo de emergencia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">desarrollo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gimnasio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mensualidad de gimnasio</t>
+    <t xml:space="preserve">fecha pago </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="mm/dd/yy"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -181,7 +201,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -194,12 +214,28 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -325,31 +361,34 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="25.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="25.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="11.4"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="0" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -357,43 +396,45 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="1" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="1" t="n">
-        <v>25000</v>
-      </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="7" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F2" s="0"/>
+      <c r="G2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="1" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="1" t="n">
+      <c r="C3" s="1" t="n">
         <v>200000</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>12</v>
-      </c>
+      <c r="D3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F3" s="0"/>
       <c r="G3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -401,19 +442,20 @@
         <v>7</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1" t="n">
         <v>14500</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="D4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F4" s="0"/>
+      <c r="G4" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -421,19 +463,22 @@
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>26300</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="1" t="n">
-        <v>26300</v>
-      </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="7" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F5" s="0" t="s">
         <v>15</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -443,98 +488,131 @@
       <c r="B6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="0" t="n">
+        <v>22000</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="1" t="n">
-        <v>30700</v>
-      </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>11</v>
+      <c r="G6" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>12000</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="C7" s="1" t="n">
+        <v>30700</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="7" t="s">
         <v>20</v>
       </c>
+      <c r="F7" s="0" t="s">
+        <v>21</v>
+      </c>
       <c r="G7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="1" t="n">
-        <v>11000</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F8" s="0"/>
       <c r="G8" s="1" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="1" t="n">
+      <c r="C9" s="1" t="n">
+        <v>11000</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F9" s="0"/>
+      <c r="G9" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="1" t="n">
         <v>200000</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="D10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F10" s="0"/>
+      <c r="G10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="0" t="n">
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="1" t="n">
         <v>70000</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>22</v>
-      </c>
+      <c r="D11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F11" s="0"/>
+      <c r="G11" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E12" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -545,4 +623,43 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>